<commit_message>
PSR-2045 & 2046 armsLength & outStanding Loans template update
</commit_message>
<xml_diff>
--- a/conf/TEMPLATE - SIPP Arms length land or property.xlsx
+++ b/conf/TEMPLATE - SIPP Arms length land or property.xlsx
@@ -9,7 +9,7 @@
   <calcPr/>
   <extLst>
     <ext uri="GoogleSheetsCustomDataVersion2">
-      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId5" roundtripDataChecksum="ioSrfQVCHqajycikeCyIA1jSCnjW1gaAc2Z0zsmQ2f0="/>
+      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId5" roundtripDataChecksum="wLVZmjLlGl//IAiszR09sJVKImfnVbODkHwVp6XTeec="/>
     </ext>
   </extLst>
 </workbook>
@@ -25,7 +25,7 @@
         <color theme="1"/>
         <sz val="11.0"/>
       </rPr>
-      <t xml:space="preserve">The questions in this section relate to a direct or indirect interest in arm's length land or property from a connected party. 
+      <t xml:space="preserve">The questions in this section relate to a direct or indirect interest in arm's length land or property. 
 </t>
     </r>
     <r>
@@ -586,7 +586,7 @@
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="1" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="top" wrapText="1"/>
+      <alignment readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
     <xf borderId="1" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="top" wrapText="1"/>

</xml_diff>